<commit_message>
SSLC debt sheet: Exos loan stands (license denied)
</commit_message>
<xml_diff>
--- a/drafts/SSLC_QB_Equity_Debt_Microcosm_Facility_2026-10-10.xlsx
+++ b/drafts/SSLC_QB_Equity_Debt_Microcosm_Facility_2026-10-10.xlsx
@@ -93,7 +93,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -115,11 +115,55 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -174,6 +218,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -604,9 +650,9 @@
           <t>EQUITY</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
+      <c r="B7" s="26" t="n"/>
+      <c r="C7" s="26" t="n"/>
+      <c r="D7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -720,9 +766,9 @@
           <t>DEBT (as of 10/2/2026)</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="27" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -835,7 +881,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>QB Acct 2720 — to be cancelled</t>
+          <t>QB Acct 2720. Loan STANDS: SSLC board denied the license, so it was not cancelled (John 10/11)</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -876,9 +922,9 @@
           <t>FACILITY COSTS (shared, 3111 Lomita Blvd)</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="27" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -992,9 +1038,9 @@
           <t>MICROCOSM OFFSET (illustrative at 50% share assumption)</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
+      <c r="B30" s="26" t="n"/>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="27" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -1417,11 +1463,11 @@
           <t>Investor / Ownership Breakdown</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+      <c r="B13" s="26" t="n"/>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="27" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1549,11 +1595,11 @@
           <t>NOTE: No SSLC cap table or stock ledger found on disk. No preferred stock. Exos investment confirmed per AAA. Founder / Microcosm shares require SSLC cap table (Eqvista or corporate records).</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="27" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1633,12 +1679,12 @@
           <t>Long-term Loans &amp; Notes</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="B3" s="26" t="n"/>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="27" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1786,7 +1832,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>11% p.a. (ROFR §3). Accrued interest ~$6,958 (not booked). To be cancelled as license consideration per Jon 10/2 decision.</t>
+          <t>11% p.a. Accrued interest ~$6,958 (not booked); ~$38,158 total at 10/2. Loan STANDS: license denied, no cancellation (John 10/11).</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1864,12 +1910,12 @@
           <t>Current Liabilities (Other)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="26" t="n"/>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="27" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -2172,12 +2218,12 @@
           <t>FY26: Jul 1, 2025 – Jun 30, 2026 (12 months, CONFIRMED from QB)</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="B3" s="26" t="n"/>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="27" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2384,12 +2430,12 @@
           <t>FY27 PARTIAL: Jul 1 – Aug 21, 2026 (52 days, CONFIRMED from QB)</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
+      <c r="B11" s="26" t="n"/>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="26" t="n"/>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="27" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -2596,12 +2642,12 @@
           <t>ESTIMATED: Aug 22 – Oct 10, 2026 (~50 days) — FY26 monthly rate proxy</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="27" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -2653,12 +2699,12 @@
           <t>2-YEAR SUMMARY (approx. Jan 2024 – Oct 2026, ~33 months)</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n"/>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="27" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
@@ -2666,8 +2712,8 @@
           <t>Jan 2024–Jun 2024 (6 mo)</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="27" t="n"/>
       <c r="D23" s="23" t="n">
         <v>176989</v>
       </c>
@@ -2689,8 +2735,8 @@
           <t>FY25: Jul 2024–Jun 2025 (12 mo)</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
+      <c r="B24" s="26" t="n"/>
+      <c r="C24" s="27" t="n"/>
       <c r="D24" s="23" t="n">
         <v>353978</v>
       </c>
@@ -2712,8 +2758,8 @@
           <t>FY26: Jul 2025–Jun 2026 (12 mo)</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
+      <c r="B25" s="26" t="n"/>
+      <c r="C25" s="27" t="n"/>
       <c r="D25" s="11" t="n">
         <v>353977.53</v>
       </c>
@@ -2735,8 +2781,8 @@
           <t>FY27: Jul 1–Aug 21, 2026 (52 days)</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
+      <c r="B26" s="26" t="n"/>
+      <c r="C26" s="27" t="n"/>
       <c r="D26" s="11" t="n">
         <v>32860.21</v>
       </c>
@@ -2758,8 +2804,8 @@
           <t>FY27: Aug 22–Oct 10, 2026 (~50 days)</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
+      <c r="B27" s="26" t="n"/>
+      <c r="C27" s="27" t="n"/>
       <c r="D27" s="23" t="n">
         <v>49163</v>
       </c>
@@ -2781,8 +2827,8 @@
           <t>TOTAL ~2-YEAR FACILITY COSTS (est.)</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
+      <c r="B28" s="26" t="n"/>
+      <c r="C28" s="27" t="n"/>
       <c r="D28" s="14" t="n">
         <v>966967.74</v>
       </c>
@@ -2804,17 +2850,17 @@
           <t>NOTE: 2-yr range interpreted as Jan 2024–Oct 2026 (~33 months). Only FY26 and FY27 partial confirmed from QB. If John means Oct 2024–Oct 2026 (24 months), remove Jan–Jun 2024 ($177K) and FY25 ($354K) rows → total confirmed+est. $702K, offset at 50% = $351K.</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
+      <c r="B29" s="26" t="n"/>
+      <c r="C29" s="26" t="n"/>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="26" t="n"/>
+      <c r="F29" s="26" t="n"/>
+      <c r="G29" s="27" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A3:G3"/>
@@ -2859,10 +2905,10 @@
           <t>INPUTS — cells in amber = management assumptions (editable)</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
+      <c r="B2" s="26" t="n"/>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="27" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -2880,8 +2926,8 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="27" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -2897,8 +2943,8 @@
           <t>MANAGEMENT ASSUMPTION — change this value. 50% = equal split. Verify against sq ft, facility lease, or cost-sharing agreement between SSLC and Microcosm.</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
+      <c r="D4" s="26" t="n"/>
+      <c r="E4" s="27" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2914,8 +2960,8 @@
           <t>Jan 2024–Oct 2026, ~33 months. Confirmed $387K + estimated $580K. See Facility Costs sheet.</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2931,8 +2977,8 @@
           <t>QB Acct 2385. Confirmed. Growing ~$500/period.</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
+      <c r="D6" s="26" t="n"/>
+      <c r="E6" s="27" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2950,8 +2996,8 @@
           <t>~33 months. John stated 'about 2 years'. Longer range used for conservatism.</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -2966,10 +3012,10 @@
           <t>CALCULATED RESULTS (sensitivity table)</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
+      <c r="B9" s="26" t="n"/>
+      <c r="C9" s="26" t="n"/>
+      <c r="D9" s="26" t="n"/>
+      <c r="E9" s="27" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -3115,10 +3161,10 @@
           <t>INTERPRETATION AND LEGAL CAVEATS</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
+      <c r="B17" s="26" t="n"/>
+      <c r="C17" s="26" t="n"/>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="27" t="n"/>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -3126,10 +3172,10 @@
           <t>At 50% share: SSLC offset claim ($483K) slightly exceeds Due to Microcosm ($451K) by ~$32K → if legally recognized, SSLC becomes net creditor.</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="27" t="n"/>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -3137,10 +3183,10 @@
           <t>At 40% share: offset ($387K) &lt; Due-to ($451K) → SSLC net-owes ~$64K after offset.</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="27" t="n"/>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -3148,10 +3194,10 @@
           <t>At 60% share: offset ($580K) &gt; Due-to ($451K) → SSLC net creditor by ~$129K.</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
+      <c r="B20" s="26" t="n"/>
+      <c r="C20" s="26" t="n"/>
+      <c r="D20" s="26" t="n"/>
+      <c r="E20" s="27" t="n"/>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
@@ -3159,10 +3205,10 @@
           <t>LEGAL BASIS REQUIRED: No written cost-sharing agreement found on disk. To assert this offset SSLC needs: (1) proof it paid 100% of shared costs; (2) a written agreement or lease provision creating Microcosm's obligation; (3) sq footage or usage basis for the share %; (4) determination whether 'Due to Microcosm' $451K is a separate loan or already includes facility charges (if the latter, double-counting occurs).</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
+      <c r="B21" s="26" t="n"/>
+      <c r="C21" s="26" t="n"/>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="27" t="n"/>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
@@ -3170,10 +3216,10 @@
           <t>[verify] FY25 QB data not on disk — estimated at FY26 rate. If actual FY25 is lower, the 2-yr total and offset decline. Pull FY25 QB P&amp;L to confirm.</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
+      <c r="B22" s="26" t="n"/>
+      <c r="C22" s="26" t="n"/>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="27" t="n"/>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
@@ -3181,18 +3227,17 @@
           <t>[verify] 'Due to Microcosm' growing ~$500/period. Determine if this is a loan facility or accruing facility charges — if the latter, the offset logic must be restructured.</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
+      <c r="B23" s="26" t="n"/>
+      <c r="C23" s="26" t="n"/>
+      <c r="D23" s="26" t="n"/>
+      <c r="E23" s="27" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="A1:E1"/>
@@ -3201,6 +3246,7 @@
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="C6:E6"/>
   </mergeCells>

</xml_diff>

<commit_message>
SSLC equity/debt: 10/11 balance sheet + cash bridge; Exos loan stands
</commit_message>
<xml_diff>
--- a/drafts/SSLC_QB_Equity_Debt_Microcosm_Facility_2026-10-10.xlsx
+++ b/drafts/SSLC_QB_Equity_Debt_Microcosm_Facility_2026-10-10.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facility Costs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Microcosm Offset" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +59,13 @@
       <i val="1"/>
       <color rgb="007B3A00"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -163,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,6 +228,7 @@
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -604,21 +613,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared: 2026-10-10  |  For: John Quinn, CEO / SSLC Board</t>
+          <t>Prepared: 2026-10-11  |  For: John Quinn, CEO / SSLC Board</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>QB SESSION EXPIRED (last live pull 10/2/2026). Browser unavailable. John must log in once to refresh. All figures from on-disk QB PDFs and board packages.</t>
+          <t>Source: QB live pull 10/11/2026 (SSLC_Balance_Sheet.xlsx + SSLC_Transaction_Detail_by_Account.xlsx).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Sources: data-room/SSLC/2026-7_BS_8-21-26.pdf  ·  data-room/SSLC/ExpensesPerformance_2025-6.pdf  ·  data-room/SSLC/2026-7_PL_8-21-26.pdf  ·  drafts/SSLC_Board_Package_2026-10-06.pdf</t>
+          <t>Sources: data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx  ·  data-room/SSLC/qb-2026-10-11/SSLC_Transaction_Detail_by_Account.xlsx</t>
         </is>
       </c>
     </row>
@@ -721,11 +730,11 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>-2571012.99</v>
+        <v>-2571013</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>QB Balance Sheet 8/21/2026</t>
+          <t>QB Balance Sheet 10/11/2026</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -737,15 +746,15 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Total Stockholders' Equity (10/2/2026)</t>
+          <t>Total Stockholders' Equity (10/11/2026)</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>-1403075</v>
+        <v>-1443882</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Board Package 10/6/2026 PDF</t>
+          <t>QB Balance Sheet 10/11/2026</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -1221,7 +1230,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
@@ -1234,7 +1243,7 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F3" s="6" t="n"/>
@@ -1247,7 +1256,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
@@ -1260,7 +1269,7 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F4" s="6" t="n"/>
@@ -1273,7 +1282,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
@@ -1284,7 +1293,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F5" s="6" t="n"/>
@@ -1297,7 +1306,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
@@ -1310,7 +1319,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F6" s="6" t="n"/>
@@ -1323,7 +1332,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C7" s="14" t="n">
@@ -1336,7 +1345,7 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F7" s="6" t="n"/>
@@ -1349,11 +1358,11 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>-2571012.99</v>
+        <v>-2571013</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
@@ -1362,7 +1371,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
@@ -1375,20 +1384,20 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>309846.15</v>
+        <v>112666</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>FY27 Q1 partial; will close to retained earnings at year-end</t>
+          <t>FY27 YTD net income through 10/11/2026</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F9" s="6" t="n"/>
@@ -1396,16 +1405,16 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>TOTAL STOCKHOLDERS' EQUITY (8/21/2026)</t>
+          <t>TOTAL STOCKHOLDERS' EQUITY (10/11/2026)</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>8/21/2026</t>
+          <t>10/11/2026</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>-1246701.84</v>
+        <v>-1443882</v>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
@@ -1414,7 +1423,7 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>QB BS (data-room/2026-7_BS_8-21-26.pdf)</t>
+          <t>QB BS (data-room/SSLC/qb-2026-10-11/SSLC_Balance_Sheet.xlsx)</t>
         </is>
       </c>
       <c r="F10" s="6" t="n"/>
@@ -1422,7 +1431,7 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>TOTAL STOCKHOLDERS' EQUITY (10/2/2026, latest)</t>
+          <t>TOTAL STOCKHOLDERS' EQUITY (10/2/2026, prior period)</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -1435,7 +1444,7 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>From board package; QB equity detail above is 8/21 (latest QB pull on disk)</t>
+          <t>Prior period; 10/11/2026 figure above supersedes this.</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -3252,4 +3261,292 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>10/2 → 10/11 Cash Bridge</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Amount ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Beginning cash (10/2/2026)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>198419</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>INFLOWS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-86 (10/7)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>142605.55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-87 (10/7)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>200700</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-88 (10/7)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>78115</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total AR collections (per GL, EFT1007)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>421420.55</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>OUTFLOWS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vendor payables Bill.com — Hexcel Corp (10/5, JE 270131)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-11091.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vendor payables Bill.com — Ileana Intl + Stratus (10/6, JE 270135)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-3316</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Chase Amazon VISA partial payment (10/5, EFT1005)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LACFD permit / hazardous waste (10/2, CK4488)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-2452</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hartford Life insurance (10/8, EFT1008)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>-1029.56</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Empower 401K + benefits (10/9, EFT1009)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>-1730.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fidelity 401K (10/9, CK4489)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paychex payroll admin (10/9, EFT1009)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>-229.39</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total outflows (per GL)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>-30349.15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>NET CHANGE PER GL</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>391071.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rounding / beginning-balance adjustment</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>854.05</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Ending cash (10/11/2026)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>590344.45</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Source: SSLC_Transaction_Detail_by_Account.xlsx (qb-2026-10-11)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>All collections from Intuitive Machines (Acct 1100 AR Billed → 1030 Checking).</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>No AR Unbilled (1110) activity between 10/2–10/11 — no new billing-ahead entries recorded.</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>$854 rounding gap reflects that stated beginning of $198,419 is rounded; GL-derived net = $391,071.</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>